<commit_message>
Beispiel-Excel: Spalte Geschlecht ergänzt, Hinweise an v1.4.0 angepasst
</commit_message>
<xml_diff>
--- a/beispiel/Beispiel-Teilnehmer-20.xlsx
+++ b/beispiel/Beispiel-Teilnehmer-20.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Hinweise" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Teilnehmer!$A$1:$F$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Teilnehmer!$A$1:$G$21</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,15 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,9 +417,12 @@
         <v>Altersklasse</v>
       </c>
       <c r="E1" t="str">
+        <v>Geschlecht</v>
+      </c>
+      <c r="F1" t="str">
         <v>Gewichtsklasse</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Jahrgang</v>
       </c>
     </row>
@@ -445,9 +440,12 @@
         <v>U11</v>
       </c>
       <c r="E2" t="str">
+        <v>m</v>
+      </c>
+      <c r="F2" t="str">
         <v>-28 kg</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>2016</v>
       </c>
     </row>
@@ -465,9 +463,12 @@
         <v>U11</v>
       </c>
       <c r="E3" t="str">
+        <v>w</v>
+      </c>
+      <c r="F3" t="str">
         <v>-28 kg</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>2016</v>
       </c>
     </row>
@@ -485,9 +486,12 @@
         <v>U11</v>
       </c>
       <c r="E4" t="str">
+        <v>m</v>
+      </c>
+      <c r="F4" t="str">
         <v>-28 kg</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>2017</v>
       </c>
     </row>
@@ -505,9 +509,12 @@
         <v>U11</v>
       </c>
       <c r="E5" t="str">
+        <v>w</v>
+      </c>
+      <c r="F5" t="str">
         <v>-28 kg</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>2016</v>
       </c>
     </row>
@@ -525,9 +532,12 @@
         <v>U11</v>
       </c>
       <c r="E6" t="str">
+        <v>m</v>
+      </c>
+      <c r="F6" t="str">
         <v>-31 kg</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>2016</v>
       </c>
     </row>
@@ -545,9 +555,12 @@
         <v>U11</v>
       </c>
       <c r="E7" t="str">
+        <v>w</v>
+      </c>
+      <c r="F7" t="str">
         <v>-31 kg</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>2017</v>
       </c>
     </row>
@@ -565,9 +578,12 @@
         <v>U11</v>
       </c>
       <c r="E8" t="str">
+        <v>m</v>
+      </c>
+      <c r="F8" t="str">
         <v>-31 kg</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>2016</v>
       </c>
     </row>
@@ -585,9 +601,12 @@
         <v>U11</v>
       </c>
       <c r="E9" t="str">
+        <v>w</v>
+      </c>
+      <c r="F9" t="str">
         <v>-31 kg</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>2016</v>
       </c>
     </row>
@@ -605,9 +624,12 @@
         <v>U13</v>
       </c>
       <c r="E10" t="str">
+        <v>m</v>
+      </c>
+      <c r="F10" t="str">
         <v>-34 kg</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>2014</v>
       </c>
     </row>
@@ -625,9 +647,12 @@
         <v>U13</v>
       </c>
       <c r="E11" t="str">
+        <v>w</v>
+      </c>
+      <c r="F11" t="str">
         <v>-34 kg</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>2015</v>
       </c>
     </row>
@@ -645,9 +670,12 @@
         <v>U13</v>
       </c>
       <c r="E12" t="str">
+        <v>m</v>
+      </c>
+      <c r="F12" t="str">
         <v>-34 kg</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>2014</v>
       </c>
     </row>
@@ -665,9 +693,12 @@
         <v>U13</v>
       </c>
       <c r="E13" t="str">
+        <v>w</v>
+      </c>
+      <c r="F13" t="str">
         <v>-34 kg</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>2014</v>
       </c>
     </row>
@@ -685,9 +716,12 @@
         <v>U13</v>
       </c>
       <c r="E14" t="str">
+        <v>m</v>
+      </c>
+      <c r="F14" t="str">
         <v>-40 kg</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>2014</v>
       </c>
     </row>
@@ -705,9 +739,12 @@
         <v>U13</v>
       </c>
       <c r="E15" t="str">
+        <v>w</v>
+      </c>
+      <c r="F15" t="str">
         <v>-40 kg</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>2015</v>
       </c>
     </row>
@@ -725,9 +762,12 @@
         <v>U13</v>
       </c>
       <c r="E16" t="str">
+        <v>m</v>
+      </c>
+      <c r="F16" t="str">
         <v>-40 kg</v>
       </c>
-      <c r="F16">
+      <c r="G16">
         <v>2014</v>
       </c>
     </row>
@@ -745,9 +785,12 @@
         <v>U13</v>
       </c>
       <c r="E17" t="str">
+        <v>w</v>
+      </c>
+      <c r="F17" t="str">
         <v>-40 kg</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <v>2014</v>
       </c>
     </row>
@@ -765,9 +808,12 @@
         <v>U13</v>
       </c>
       <c r="E18" t="str">
+        <v>m</v>
+      </c>
+      <c r="F18" t="str">
         <v>-40 kg</v>
       </c>
-      <c r="F18">
+      <c r="G18">
         <v>2015</v>
       </c>
     </row>
@@ -785,9 +831,12 @@
         <v>U15</v>
       </c>
       <c r="E19" t="str">
+        <v>m</v>
+      </c>
+      <c r="F19" t="str">
         <v>-46 kg</v>
       </c>
-      <c r="F19">
+      <c r="G19">
         <v>2012</v>
       </c>
     </row>
@@ -805,9 +854,12 @@
         <v>U15</v>
       </c>
       <c r="E20" t="str">
+        <v>m</v>
+      </c>
+      <c r="F20" t="str">
         <v>-46 kg</v>
       </c>
-      <c r="F20">
+      <c r="G20">
         <v>2012</v>
       </c>
     </row>
@@ -825,23 +877,26 @@
         <v>U15</v>
       </c>
       <c r="E21" t="str">
+        <v>m</v>
+      </c>
+      <c r="F21" t="str">
         <v>-46 kg</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>2013</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F21"/>
+  <autoFilter ref="A1:G21"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <cols>
     <col min="1" max="1" width="105.83203125" customWidth="1"/>
   </cols>
@@ -868,7 +923,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Danach rechts bei „Teilnehmer“: „Alle Gruppen: Jeder gegen jeden“ erzeugt 31 Kämpfe.</v>
+        <v>Danach rechts bei „Teilnehmer“: „Kampflisten aller Gruppen erzeugen“ – bei 3 bis 5 Kämpfern schlägt Hajime „Jeder gegen jeden“ vor, das ergibt 31 Kämpfe.</v>
       </c>
     </row>
     <row r="6">
@@ -878,12 +933,17 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Die Spalte „Geschlecht“ (m / w / d) ist optional – hier 12 Jungen und 8 Mädchen. Ist unter Einstellungen „Nach Geschlecht trennen“ eingeschaltet, bildet Hajime getrennte Gruppen (z. B. „U11 w -28 kg“). Bei so wenigen Teilnehmern werden die Gruppen dann klein; zwei Kämpfer tragen Best of Three aus.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Die Spalte „Jahrgang“ ist nur zur Info und wird beim Import ignoriert.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>